<commit_message>
enhancement  environment test, report, configuration, and dependency
</commit_message>
<xml_diff>
--- a/data/DataUser.xlsx
+++ b/data/DataUser.xlsx
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>EMAIL</t>
   </si>
@@ -48,6 +48,30 @@
   </si>
   <si>
     <t>Of3%BGOK</t>
+  </si>
+  <si>
+    <t>sheena.jacobi@gmail.com</t>
+  </si>
+  <si>
+    <t>Hu7@7LD&amp;</t>
+  </si>
+  <si>
+    <t>creola.vandervort@gmail.com</t>
+  </si>
+  <si>
+    <t>Aq0%3MHB</t>
+  </si>
+  <si>
+    <t>reid.cartwright@hotmail.com</t>
+  </si>
+  <si>
+    <t>Qs6#pb%t</t>
+  </si>
+  <si>
+    <t>claude.walter@yahoo.com</t>
+  </si>
+  <si>
+    <t>Mo0^f1ZG</t>
   </si>
 </sst>
 </file>
@@ -420,7 +444,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{290CBC4D-1AFC-4B6D-8F9B-23F8520A0F28}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1">
@@ -439,6 +463,38 @@
         <v>3</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>